<commit_message>
completed lookup st.dialog() for claim summary on overview page; begun reorganizing helper functions and reformatting global functions for loading variables and data on most pages
</commit_message>
<xml_diff>
--- a/utilities/excel/short_list.xlsx
+++ b/utilities/excel/short_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\banghamf\Documents\claims_automation\utilities\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC366E19-C1B3-4C82-BD07-A2B95D47ABCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C4EC028-D695-425F-AC44-F653592A5DAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="short_list_claims" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="22">
   <si>
     <t>CCR#</t>
   </si>
@@ -32,9 +32,6 @@
     <t>Assigned_Date</t>
   </si>
   <si>
-    <t>cocciaka</t>
-  </si>
-  <si>
     <t>test_user</t>
   </si>
   <si>
@@ -44,6 +41,9 @@
     <t>test_user2</t>
   </si>
   <si>
+    <t>branonem</t>
+  </si>
+  <si>
     <t>Update_Date</t>
   </si>
   <si>
@@ -53,18 +53,6 @@
     <t>Update_Notes</t>
   </si>
   <si>
-    <t>Pending Quote Approval</t>
-  </si>
-  <si>
-    <t>This is a test update</t>
-  </si>
-  <si>
-    <t>This is another update test.</t>
-  </si>
-  <si>
-    <t>This is another another update test.</t>
-  </si>
-  <si>
     <t>Assigned for Evaluation</t>
   </si>
   <si>
@@ -89,10 +77,16 @@
     <t>THIS IS THE LAST TEST</t>
   </si>
   <si>
-    <t>we should probably hold off on the updates for at least a little while.</t>
-  </si>
-  <si>
     <t>progress baby</t>
+  </si>
+  <si>
+    <t>Pending CAR Completion</t>
+  </si>
+  <si>
+    <t>This was brought up in last meeting; appears to be quite old</t>
+  </si>
+  <si>
+    <t>Should follow up on this during this weeks meeting</t>
   </si>
 </sst>
 </file>
@@ -459,46 +453,46 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>107466</v>
+        <v>123456</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="1">
-        <v>46198</v>
+        <v>46259</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>123456</v>
+        <v>123123</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>
       </c>
       <c r="C3" s="1">
-        <v>46259</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>123123</v>
+        <v>654321</v>
       </c>
       <c r="B4" t="s">
         <v>5</v>
       </c>
       <c r="C4" s="1">
-        <v>46228</v>
+        <v>46246</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>654321</v>
+        <v>105376</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
       </c>
       <c r="C5" s="1">
-        <v>46246</v>
+        <v>45957</v>
       </c>
     </row>
   </sheetData>
@@ -508,12 +502,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.5703125" customWidth="1"/>
-    <col min="4" max="4" width="63.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -532,7 +525,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>107466</v>
+        <v>123456</v>
       </c>
       <c r="B2" s="1">
         <v>46282</v>
@@ -546,7 +539,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>107466</v>
+        <v>123456</v>
       </c>
       <c r="B3" s="1">
         <v>46282</v>
@@ -560,7 +553,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>107466</v>
+        <v>123456</v>
       </c>
       <c r="B4" s="1">
         <v>46282</v>
@@ -574,7 +567,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>123456</v>
+        <v>123123</v>
       </c>
       <c r="B5" s="1">
         <v>46282</v>
@@ -588,7 +581,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>123456</v>
+        <v>123123</v>
       </c>
       <c r="B6" s="1">
         <v>46282</v>
@@ -602,13 +595,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>123456</v>
+        <v>654321</v>
       </c>
       <c r="B7" s="1">
         <v>46282</v>
       </c>
       <c r="C7" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D7" t="s">
         <v>17</v>
@@ -616,27 +609,27 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>123123</v>
+        <v>123456</v>
       </c>
       <c r="B8" s="1">
         <v>46282</v>
       </c>
       <c r="C8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" t="s">
         <v>18</v>
-      </c>
-      <c r="D8" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>123123</v>
+        <v>105376</v>
       </c>
       <c r="B9" s="1">
-        <v>46282</v>
+        <v>46295</v>
       </c>
       <c r="C9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D9" t="s">
         <v>20</v>
@@ -644,44 +637,16 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>654321</v>
-      </c>
-      <c r="B10" s="1">
-        <v>46282</v>
+        <v>105376</v>
+      </c>
+      <c r="B10" s="2">
+        <v>46295</v>
       </c>
       <c r="C10" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="D10" t="s">
         <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>107466</v>
-      </c>
-      <c r="B11" s="2">
-        <v>46282</v>
-      </c>
-      <c r="C11" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>123456</v>
-      </c>
-      <c r="B12" s="2">
-        <v>46282</v>
-      </c>
-      <c r="C12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>